<commit_message>
data: update Project Dashboard Dataset.xlsx database records
</commit_message>
<xml_diff>
--- a/backend/Project Dashboard Dataset.xlsx
+++ b/backend/Project Dashboard Dataset.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2202A5B3-B9B3-4EE3-9362-380F2CB0B21F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4BC0F65-FAEB-4CAB-9E8D-A5AB2C185C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$P$326</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2466,8 +2465,8 @@
     <col min="4" max="4" width="36.36328125" style="13" customWidth="1"/>
     <col min="5" max="5" width="13.26953125" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.453125" style="14" customWidth="1"/>
-    <col min="7" max="7" width="8.7265625" style="12" customWidth="1"/>
-    <col min="8" max="8" width="11.26953125" style="12" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" style="12" customWidth="1"/>
+    <col min="8" max="8" width="18.1796875" style="12" customWidth="1"/>
     <col min="9" max="9" width="10.6328125" style="21" customWidth="1"/>
     <col min="10" max="10" width="14.1796875" style="13" customWidth="1"/>
     <col min="11" max="11" width="25" style="13" customWidth="1"/>
@@ -5470,7 +5469,7 @@
       <c r="O71" s="8"/>
       <c r="P71" s="8"/>
     </row>
-    <row r="72" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="6" t="s">
         <v>511</v>
       </c>
@@ -5512,7 +5511,7 @@
       <c r="O72" s="8"/>
       <c r="P72" s="8"/>
     </row>
-    <row r="73" spans="1:16" ht="4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="6" t="s">
         <v>512</v>
       </c>

</xml_diff>